<commit_message>
updated columns feature 7
</commit_message>
<xml_diff>
--- a/OrgSight_Feature_Tracker.xlsx
+++ b/OrgSight_Feature_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itinfoalvarezandmarsalind-my.sharepoint.com/personal/jagritjain_alvarezandmarsal_com/Documents/Documents/APPS/ORG_ANALYSIS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96C79565-2483-4461-A3B3-104C378EC6FE}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{376379D9-6AAC-4CA4-902E-6EB43057BC84}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="124">
   <si>
     <t>OrgSight  |  Feature Development Tracker</t>
   </si>
@@ -179,9 +179,6 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>Formula parser + column renderer needed. Scope: basic arithmetic &amp; IF logic.</t>
-  </si>
-  <si>
     <t>Properties Cleaning Heatmap</t>
   </si>
   <si>
@@ -402,6 +399,18 @@
   </si>
   <si>
     <t>Fixes known OrgVue gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right now : a Formula Editor panel in the workspace where you can write simple math expressions referencing any column in your dataset:
+Cost per FTE    =  FLC / FTE
+Annual Cost     =  Monthly_Salary * 12
+Total Comp      =  Base_Salary + Bonus + Benefits
+Cost Ratio      =  FLC / Total_Budget * 100
+Supports: +, -, *, /, parentheses, and numeric literals. As you type the expression, a live preview evaluates it against the first record so you can see the result instantly. If the expression is invalid (e.g., references a column that doesn't exist), you see a red error message inline.
+</t>
+  </si>
+  <si>
+    <t>Define the scope - to expand or not? (IF conditional logic)</t>
   </si>
 </sst>
 </file>
@@ -688,9 +697,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -713,6 +719,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1345,15 +1354,17 @@
       <c r="E13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>48</v>
+      <c r="F13" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="11" t="s">
+        <v>122</v>
+      </c>
       <c r="I13" s="11" t="s">
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
@@ -1367,23 +1378,23 @@
         <v>44</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="E14" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>48</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J14" s="11"/>
       <c r="K14" s="11"/>
@@ -1397,13 +1408,13 @@
         <v>44</v>
       </c>
       <c r="C15" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="E15" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>48</v>
@@ -1413,7 +1424,7 @@
       </c>
       <c r="H15" s="11"/>
       <c r="I15" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
@@ -1435,7 +1446,7 @@
     </row>
     <row r="17" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" s="29"/>
       <c r="C17" s="29"/>
@@ -1454,16 +1465,16 @@
         <v>10</v>
       </c>
       <c r="B18" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="D18" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="E18" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>63</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>48</v>
@@ -1473,7 +1484,7 @@
       </c>
       <c r="H18" s="16"/>
       <c r="I18" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J18" s="16"/>
       <c r="K18" s="16"/>
@@ -1484,26 +1495,26 @@
         <v>11</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C19" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="E19" s="16" t="s">
         <v>66</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>67</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>48</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J19" s="16"/>
       <c r="K19" s="16"/>
@@ -1543,8 +1554,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
-        <v>69</v>
+      <c r="A1" s="36" t="s">
+        <v>68</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -1555,8 +1566,8 @@
       <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
-        <v>70</v>
+      <c r="A2" s="34" t="s">
+        <v>69</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
@@ -1567,43 +1578,43 @@
       <c r="H2" s="29"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="34" t="s">
+      <c r="E4" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="F4" s="42" t="s">
         <v>73</v>
       </c>
-      <c r="F4" s="34" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="40" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="41" t="s">
+      <c r="B5" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="C5" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="D5" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="E5" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="E5" s="42" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" s="39" t="s">
-        <v>78</v>
+      <c r="F5" s="38" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1612,7 +1623,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>3</v>
@@ -1624,7 +1635,7 @@
         <v>8</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1632,7 +1643,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>15</v>
@@ -1692,7 +1703,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>15</v>
@@ -1752,7 +1763,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C15" s="21" t="s">
         <v>44</v>
@@ -1772,7 +1783,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C16" s="21" t="s">
         <v>44</v>
@@ -1781,10 +1792,10 @@
         <v>48</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1792,7 +1803,7 @@
         <v>9</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>44</v>
@@ -1804,7 +1815,7 @@
         <v>25</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1812,10 +1823,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>48</v>
@@ -1824,7 +1835,7 @@
         <v>25</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1832,19 +1843,19 @@
         <v>11</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1883,8 +1894,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
-        <v>88</v>
+      <c r="A1" s="36" t="s">
+        <v>87</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -1894,8 +1905,8 @@
       <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
-        <v>89</v>
+      <c r="A2" s="34" t="s">
+        <v>88</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
@@ -1907,163 +1918,163 @@
     <row r="3" spans="1:7" ht="8" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="C4" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="D4" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="E4" s="17" t="s">
         <v>93</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>94</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="C5" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="D5" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="E5" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="F5" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="G5" s="25" t="s">
         <v>101</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C6" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="E6" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="F6" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="27" t="s">
         <v>106</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="D7" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="E7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="G7" s="25" t="s">
         <v>110</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="G7" s="25" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="D8" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="E8" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="G8" s="27" t="s">
         <v>114</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="G8" s="27" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B9" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="D9" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="E9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="G9" s="25" t="s">
         <v>118</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C10" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="E10" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="G10" s="27" t="s">
         <v>121</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
summary and phasing improved+ multi-select move
</commit_message>
<xml_diff>
--- a/OrgSight_Feature_Tracker.xlsx
+++ b/OrgSight_Feature_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itinfoalvarezandmarsalind-my.sharepoint.com/personal/jagritjain_alvarezandmarsal_com/Documents/Documents/APPS/ORG_ANALYSIS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{376379D9-6AAC-4CA4-902E-6EB43057BC84}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F4FC275-7C88-450C-8F8C-CD41A6ABA19B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1386,8 +1386,8 @@
       <c r="E14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>48</v>
+      <c r="F14" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="G14" s="13" t="s">
         <v>52</v>
@@ -1768,8 +1768,8 @@
       <c r="C15" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="12" t="s">
-        <v>48</v>
+      <c r="D15" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
pills update on org details
</commit_message>
<xml_diff>
--- a/OrgSight_Feature_Tracker.xlsx
+++ b/OrgSight_Feature_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itinfoalvarezandmarsalind-my.sharepoint.com/personal/jagritjain_alvarezandmarsal_com/Documents/Documents/APPS/ORG_ANALYSIS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E8D098A-6BC6-474E-AAB2-878F2F177767}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_EBBDD73C6D5A272E4D7A8B3D1FD93A7099AF6BB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F219592A-0A47-420C-B691-619A7A815D35}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feature Tracker" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="86">
   <si>
     <t>OrgSight  |  Feature Development Tracker</t>
   </si>
@@ -259,16 +259,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>2</t>
-  </si>
-  <si>
-    <t>7</t>
   </si>
   <si>
     <t>Feature</t>
@@ -1233,10 +1224,10 @@
         <v>25</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
@@ -1288,7 +1279,7 @@
       <c r="E15" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="5" t="s">
         <v>19</v>
       </c>
       <c r="G15" s="7" t="s">
@@ -1401,16 +1392,6 @@
     <mergeCell ref="A12:L12"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
-  <conditionalFormatting sqref="F15">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF00B050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="F4:F25" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Completed,In Progress,Pending,On Hold,Cancelled"</formula1>
@@ -1483,20 +1464,20 @@
       <c r="A5" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="33">
+        <v>9</v>
+      </c>
+      <c r="C5" s="35">
+        <v>2</v>
+      </c>
+      <c r="D5" s="31">
+        <v>3</v>
+      </c>
+      <c r="E5" s="37">
+        <v>6</v>
+      </c>
+      <c r="F5" s="34" t="s">
         <v>75</v>
-      </c>
-      <c r="C5" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" s="34" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1505,7 +1486,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>3</v>
@@ -1517,7 +1498,7 @@
         <v>8</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1525,7 +1506,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>15</v>
@@ -1585,7 +1566,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>15</v>
@@ -1645,7 +1626,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C15" s="21" t="s">
         <v>44</v>
@@ -1685,13 +1666,13 @@
         <v>9</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="12" t="s">
-        <v>48</v>
+      <c r="D17" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>25</v>
@@ -1705,7 +1686,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C18" s="23" t="s">
         <v>59</v>
@@ -1725,7 +1706,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C19" s="23" t="s">
         <v>59</v>

</xml_diff>